<commit_message>
Añadidos, nueva columna y agarrar datos a partir de 1000 en health cost
</commit_message>
<xml_diff>
--- a/public/Formato facturacion - final.xlsx
+++ b/public/Formato facturacion - final.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Documents\S&amp;P\Documentos automatizacion\EOR\Web facturación\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7958E1-6F9D-4C34-9320-9A2B95D7AAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E196B7E-D858-4C8E-88AE-F136101039D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7C2F0237-C030-49A0-B1F1-0009A5922E79}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="INVOICING" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">INVOICING!$A$3:$BN$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">INVOICING!$A$3:$BO$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="68">
   <si>
     <t>COST REPORT</t>
   </si>
@@ -261,6 +261,9 @@
       </rPr>
       <t xml:space="preserve"> (Previous months) Breakdown</t>
     </r>
+  </si>
+  <si>
+    <t>SENA QUOTE</t>
   </si>
 </sst>
 </file>
@@ -981,7 +984,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C983BF9-744E-4096-9D6A-6BB252C9D3E3}">
-  <dimension ref="A1:BM7"/>
+  <dimension ref="A1:BN7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="7" bestFit="1" customWidth="1"/>
@@ -1014,26 +1017,26 @@
     <col min="47" max="47" width="9.5546875" style="7" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="10.44140625" style="7" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="8.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="50" max="51" width="8.88671875" style="7" customWidth="1"/>
-    <col min="52" max="52" width="9" style="7" customWidth="1"/>
-    <col min="53" max="53" width="12.5546875" style="7" customWidth="1"/>
-    <col min="54" max="54" width="11.5546875" style="7" customWidth="1"/>
-    <col min="55" max="55" width="8.44140625" style="7" customWidth="1"/>
-    <col min="56" max="56" width="8.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="7.109375" style="7" customWidth="1"/>
-    <col min="58" max="58" width="11.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="12.5546875" style="7" customWidth="1"/>
-    <col min="60" max="60" width="10.44140625" style="7" customWidth="1"/>
-    <col min="61" max="61" width="9.44140625" style="7" customWidth="1"/>
-    <col min="62" max="62" width="8.33203125" style="7" customWidth="1"/>
-    <col min="63" max="63" width="12.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="12.5546875" style="7" hidden="1" customWidth="1"/>
-    <col min="65" max="65" width="10.88671875" style="7" hidden="1" customWidth="1"/>
-    <col min="66" max="66" width="14.5546875" style="7" customWidth="1"/>
-    <col min="67" max="16384" width="9.109375" style="7"/>
+    <col min="50" max="52" width="8.88671875" style="7" customWidth="1"/>
+    <col min="53" max="53" width="9" style="7" customWidth="1"/>
+    <col min="54" max="54" width="12.5546875" style="7" customWidth="1"/>
+    <col min="55" max="55" width="11.5546875" style="7" customWidth="1"/>
+    <col min="56" max="56" width="8.44140625" style="7" customWidth="1"/>
+    <col min="57" max="57" width="8.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="7.109375" style="7" customWidth="1"/>
+    <col min="59" max="59" width="11.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5546875" style="7" customWidth="1"/>
+    <col min="61" max="61" width="10.44140625" style="7" customWidth="1"/>
+    <col min="62" max="62" width="9.44140625" style="7" customWidth="1"/>
+    <col min="63" max="63" width="8.33203125" style="7" customWidth="1"/>
+    <col min="64" max="64" width="12.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="12.5546875" style="7" hidden="1" customWidth="1"/>
+    <col min="66" max="66" width="10.88671875" style="7" hidden="1" customWidth="1"/>
+    <col min="67" max="67" width="14.5546875" style="7" customWidth="1"/>
+    <col min="68" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:66" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
@@ -1086,8 +1089,8 @@
       <c r="AW1" s="5"/>
       <c r="AX1" s="5"/>
       <c r="AY1" s="5"/>
-      <c r="AZ1" s="6"/>
-      <c r="BA1" s="5"/>
+      <c r="AZ1" s="5"/>
+      <c r="BA1" s="6"/>
       <c r="BB1" s="5"/>
       <c r="BC1" s="5"/>
       <c r="BD1" s="5"/>
@@ -1095,11 +1098,12 @@
       <c r="BF1" s="5"/>
       <c r="BG1" s="5"/>
       <c r="BH1" s="5"/>
-      <c r="BI1" s="8"/>
-      <c r="BJ1" s="5"/>
-      <c r="BK1" s="6"/>
+      <c r="BI1" s="5"/>
+      <c r="BJ1" s="8"/>
+      <c r="BK1" s="5"/>
+      <c r="BL1" s="6"/>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -1156,12 +1160,12 @@
       <c r="AW2" s="40"/>
       <c r="AX2" s="40"/>
       <c r="AY2" s="40"/>
-      <c r="AZ2" s="41"/>
-      <c r="BA2" s="10"/>
-      <c r="BB2" s="37" t="s">
+      <c r="AZ2" s="40"/>
+      <c r="BA2" s="41"/>
+      <c r="BB2" s="10"/>
+      <c r="BC2" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="BC2" s="38"/>
       <c r="BD2" s="38"/>
       <c r="BE2" s="38"/>
       <c r="BF2" s="38"/>
@@ -1170,12 +1174,13 @@
       <c r="BI2" s="38"/>
       <c r="BJ2" s="38"/>
       <c r="BK2" s="38"/>
-      <c r="BL2" s="12" t="e">
-        <f>1/BG4</f>
+      <c r="BL2" s="38"/>
+      <c r="BM2" s="12" t="e">
+        <f>1/BH4</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:65" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:66" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>5</v>
       </c>
@@ -1325,47 +1330,50 @@
         <v>52</v>
       </c>
       <c r="AZ3" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="BA3" s="17"/>
-      <c r="BB3" s="16" t="s">
+      <c r="BB3" s="17"/>
+      <c r="BC3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="BC3" s="16" t="s">
+      <c r="BD3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="BD3" s="16" t="s">
+      <c r="BE3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="BE3" s="16" t="s">
+      <c r="BF3" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BF3" s="16" t="s">
+      <c r="BG3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="BG3" s="16" t="s">
+      <c r="BH3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="BH3" s="16" t="s">
+      <c r="BI3" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="BI3" s="16" t="s">
+      <c r="BJ3" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="BJ3" s="16" t="s">
+      <c r="BK3" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="BK3" s="16" t="s">
+      <c r="BL3" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="BL3" s="16" t="s">
+      <c r="BM3" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="BM3" s="16" t="s">
+      <c r="BN3" s="16" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A4" s="18"/>
       <c r="B4" s="18"/>
       <c r="C4" s="18"/>
@@ -1428,55 +1436,56 @@
       <c r="AW4" s="22"/>
       <c r="AX4" s="22"/>
       <c r="AY4" s="22"/>
-      <c r="AZ4" s="26">
-        <f t="shared" ref="AZ4" si="4">SUM($AU4:$AY4)</f>
-        <v>0</v>
-      </c>
-      <c r="BA4" s="24"/>
-      <c r="BB4" s="22">
-        <f t="shared" ref="BB4" si="5">SUM($AF4,$AN4,$AS4,$AZ4)+BD4</f>
-        <v>0</v>
-      </c>
+      <c r="AZ4" s="22"/>
+      <c r="BA4" s="26">
+        <f t="shared" ref="BA4" si="4">SUM($AU4:$AY4)</f>
+        <v>0</v>
+      </c>
+      <c r="BB4" s="24"/>
       <c r="BC4" s="22">
-        <f t="shared" ref="BC4" si="6">120*$BG4</f>
+        <f t="shared" ref="BC4" si="5">SUM($AF4,$AN4,$AS4,$BA4)+BE4</f>
         <v>0</v>
       </c>
       <c r="BD4" s="22">
-        <f t="shared" ref="BD4" si="7">SUM($AF4,$AN4,$AS4,$AZ4)*0.4%</f>
+        <f t="shared" ref="BD4" si="6">120*$BH4</f>
         <v>0</v>
       </c>
       <c r="BE4" s="22">
-        <f t="shared" ref="BE4" si="8">$BC4*19%</f>
+        <f t="shared" ref="BE4" si="7">SUM($AF4,$AN4,$AS4,$BA4)*0.4%</f>
         <v>0</v>
       </c>
       <c r="BF4" s="22">
-        <f>SUM(BB4,BC4,BE4)</f>
-        <v>0</v>
-      </c>
-      <c r="BG4" s="27"/>
-      <c r="BH4" s="28" t="e">
-        <f t="shared" ref="BH4" si="9">ROUND($BB4/$BG4,2)</f>
+        <f t="shared" ref="BF4" si="8">$BD4*19%</f>
+        <v>0</v>
+      </c>
+      <c r="BG4" s="22">
+        <f>SUM(BC4,BD4,BF4)</f>
+        <v>0</v>
+      </c>
+      <c r="BH4" s="27"/>
+      <c r="BI4" s="28" t="e">
+        <f t="shared" ref="BI4" si="9">ROUND($BC4/$BH4,2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BI4" s="28" t="e">
-        <f t="shared" ref="BI4" si="10">ROUND($BC4/$BG4,2)</f>
+      <c r="BJ4" s="28" t="e">
+        <f t="shared" ref="BJ4" si="10">ROUND($BD4/$BH4,2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BJ4" s="28" t="e">
-        <f t="shared" ref="BJ4" si="11">ROUND($BE4/$BG4,2)</f>
+      <c r="BK4" s="28" t="e">
+        <f t="shared" ref="BK4" si="11">ROUND($BF4/$BH4,2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BK4" s="28" t="e">
-        <f t="shared" ref="BK4" si="12">SUM($BH4:$BJ4)</f>
+      <c r="BL4" s="28" t="e">
+        <f t="shared" ref="BL4" si="12">SUM($BI4:$BK4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BL4" s="29"/>
-      <c r="BM4" s="28" t="e">
-        <f t="shared" ref="BM4" si="13">BK4-BL4</f>
+      <c r="BM4" s="29"/>
+      <c r="BN4" s="28" t="e">
+        <f t="shared" ref="BN4" si="13">BL4-BM4</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A5" s="30"/>
       <c r="B5" s="30"/>
       <c r="C5" s="30" t="s">
@@ -1620,7 +1629,7 @@
       </c>
       <c r="AT5" s="33"/>
       <c r="AU5" s="32">
-        <f t="shared" ref="AU5:AZ5" si="16">SUM(AU4:AU4)</f>
+        <f t="shared" ref="AU5:BA5" si="16">SUM(AU4:AU4)</f>
         <v>0</v>
       </c>
       <c r="AV5" s="32">
@@ -1639,15 +1648,12 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="AZ5" s="32">
+      <c r="AZ5" s="32"/>
+      <c r="BA5" s="32">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="BA5" s="24"/>
-      <c r="BB5" s="32">
-        <f>SUM(BB4:BB4)</f>
-        <v>0</v>
-      </c>
+      <c r="BB5" s="24"/>
       <c r="BC5" s="32">
         <f>SUM(BC4:BC4)</f>
         <v>0</v>
@@ -1664,11 +1670,11 @@
         <f>SUM(BF4:BF4)</f>
         <v>0</v>
       </c>
-      <c r="BG5" s="32"/>
-      <c r="BH5" s="34" t="e">
-        <f>SUM(BH4:BH4)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="BG5" s="32">
+        <f>SUM(BG4:BG4)</f>
+        <v>0</v>
+      </c>
+      <c r="BH5" s="32"/>
       <c r="BI5" s="34" t="e">
         <f>SUM(BI4:BI4)</f>
         <v>#DIV/0!</v>
@@ -1681,13 +1687,17 @@
         <f>SUM(BK4:BK4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BL5" s="29"/>
-      <c r="BM5" s="28" t="e">
-        <f>BK5-BL5</f>
+      <c r="BL5" s="34" t="e">
+        <f>SUM(BL4:BL4)</f>
         <v>#DIV/0!</v>
       </c>
+      <c r="BM5" s="29"/>
+      <c r="BN5" s="28" t="e">
+        <f>BL5-BM5</f>
+        <v>#DIV/0!</v>
+      </c>
     </row>
-    <row r="7" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A7" s="35" t="s">
         <v>66</v>
       </c>
@@ -1697,8 +1707,8 @@
   <mergeCells count="4">
     <mergeCell ref="AH2:AN2"/>
     <mergeCell ref="AP2:AR2"/>
-    <mergeCell ref="AU2:AZ2"/>
-    <mergeCell ref="BB2:BK2"/>
+    <mergeCell ref="AU2:BA2"/>
+    <mergeCell ref="BC2:BL2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>